<commit_message>
detect empty annotation table row(s)
</commit_message>
<xml_diff>
--- a/tests/fixtures/02-Fails-03/assays/RNASeq/isa.assay.xlsx
+++ b/tests/fixtures/02-Fails-03/assays/RNASeq/isa.assay.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="143">
   <si>
     <t>Input [Sample Name]</t>
   </si>
@@ -376,9 +376,6 @@
   </si>
   <si>
     <t>Assay Title</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Assay Description</t>
@@ -484,15 +481,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
   </cellXfs>
@@ -670,8 +664,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:W7" displayName="annotationTable0" name="annotationTable0" id="2" totalsRowShown="0">
-  <autoFilter ref="A1:W7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:W9" displayName="annotationTable0" name="annotationTable0" id="2" totalsRowShown="0">
+  <autoFilter ref="A1:W9">
     <filterColumn hiddenButton="1" colId="0"/>
     <filterColumn hiddenButton="1" colId="1"/>
     <filterColumn hiddenButton="1" colId="2"/>
@@ -1062,9 +1056,9 @@
   <cols>
     <col min="1" max="1" style="2" width="28.862142857142857" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="2" width="32.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
@@ -1091,107 +1085,89 @@
       <c r="A3" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>120</v>
-      </c>
+      <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
       <c r="A4" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="B4" s="3" t="s">
         <v>120</v>
       </c>
+      <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
       <c r="A5" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
       <c r="A6" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
       <c r="A7" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>123</v>
+      </c>
+      <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
       <c r="A8" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
       <c r="A9" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>125</v>
+      </c>
+      <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
       <c r="A10" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
       <c r="A11" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
       <c r="A12" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>130</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -1199,7 +1175,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
       <c r="A13" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -1208,41 +1184,25 @@
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
       <c r="A14" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>131</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
       <c r="A15" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
       <c r="A16" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -1251,29 +1211,25 @@
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
       <c r="A17" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>134</v>
+      </c>
+      <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
       <c r="A18" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>135</v>
+      </c>
+      <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
       <c r="A19" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1282,92 +1238,52 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
       <c r="A20" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25">
       <c r="A21" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>138</v>
+      </c>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25">
       <c r="A22" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25">
       <c r="A23" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25">
       <c r="A24" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>120</v>
-      </c>
+        <v>141</v>
+      </c>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="17.25">
       <c r="A25" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1384,32 +1300,32 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:W9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
@@ -1872,6 +1788,56 @@
       <c r="W7" s="1" t="s">
         <v>70</v>
       </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="1"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="1"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="1"/>
+      <c r="W8" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="1"/>
+      <c r="R9" s="1"/>
+      <c r="S9" s="1"/>
+      <c r="T9" s="1"/>
+      <c r="U9" s="1"/>
+      <c r="V9" s="1"/>
+      <c r="W9" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1889,44 +1855,44 @@
   <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="34" max="34" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="35" max="35" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="36" max="36" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="37" max="37" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="38" max="38" style="2" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="36" max="36" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="37" max="37" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="38" max="38" style="2" width="12.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">

</xml_diff>